<commit_message>
cây quyết định v1
</commit_message>
<xml_diff>
--- a/Folder project/LenhSQL-2/Danh sách các xã thuộc VN.xlsx
+++ b/Folder project/LenhSQL-2/Danh sách các xã thuộc VN.xlsx
@@ -1,22 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f49e212d2fc23069/Documents/File ptit/Kho DL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f49e212d2fc23069/Documents/File ptit/Kho DL/Folder project/LenhSQL-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{F3096839-0868-4056-909A-8215908AE35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D1BE3E0-E891-4AA2-917B-79D7188F3045}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{F3096839-0868-4056-909A-8215908AE35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA1BFF5B-F206-4189-A9FD-0E0E2B8235AE}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{4CC679F3-2BAE-4E9F-8FFA-759A49459841}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" xr2:uid="{4CC679F3-2BAE-4E9F-8FFA-759A49459841}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
     <sheet name="Trang_tính3" sheetId="3" r:id="rId2"/>
     <sheet name="danh sách tên phố" sheetId="4" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v5.0" hidden="1">Trang_tính1!$A$1</definedName>
+    <definedName name="_xlchart.v5.1" hidden="1">Trang_tính1!$A$2:$A$2622</definedName>
+    <definedName name="_xlchart.v5.2" hidden="1">Trang_tính1!$B$1</definedName>
+    <definedName name="_xlchart.v5.3" hidden="1">Trang_tính1!$B$2:$B$2622</definedName>
+    <definedName name="_xlchart.v5.4" hidden="1">Trang_tính1!$B$1:$B$2600</definedName>
+    <definedName name="_xlchart.v5.5" hidden="1">Trang_tính1!$B$2600</definedName>
+    <definedName name="_xlchart.v5.6" hidden="1">Trang_tính1!$B$2601</definedName>
+    <definedName name="_xlchart.v5.7" hidden="1">Trang_tính1!$B$1:$B$2600</definedName>
+    <definedName name="_xlchart.v5.8" hidden="1">Trang_tính1!$B$2600</definedName>
+    <definedName name="_xlchart.v5.9" hidden="1">Trang_tính1!$B$2601</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">

</xml_diff>